<commit_message>
Atualizar LISTA.xlsx pelo Azure DevOps
</commit_message>
<xml_diff>
--- a/LISTA.xlsx
+++ b/LISTA.xlsx
@@ -663,7 +663,11 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>V.01 R.04</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Promob\Wonder Squad</t>

</xml_diff>